<commit_message>
Add interactive Plotly Dash dashboard with JSE, crypto and sentiment
</commit_message>
<xml_diff>
--- a/jse_report.xlsx
+++ b/jse_report.xlsx
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 17:49:18</t>
+          <t>2026-05-05 22:42:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 17:49:21</t>
+          <t>2026-05-05 22:42:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-05 17:49:23</t>
+          <t>2026-05-05 22:42:12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -543,7 +543,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-05 17:49:24</t>
+          <t>2026-05-05 22:42:12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-05 17:49:25</t>
+          <t>2026-05-05 22:42:13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>